<commit_message>
Protect lists in Excel for Forms3 excel template
</commit_message>
<xml_diff>
--- a/data/Excel/3.2.xlsx
+++ b/data/Excel/3.2.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="11535" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="11535"/>
   </bookViews>
   <sheets>
     <sheet name="Форма 3.0" sheetId="1" r:id="rId1"/>
@@ -2458,6 +2458,35 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="0" fillId="4" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -2482,10 +2511,6 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
@@ -2498,32 +2523,7 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="4" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="49" fontId="0" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
@@ -3091,7 +3091,7 @@
       <c r="I37" s="12"/>
     </row>
   </sheetData>
-  <sheetProtection formatRows="0" insertRows="0" deleteRows="0" selectLockedCells="1"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="RKVYkFqxXXh5cxT0sNZvExR23eZ5Inp+Vf1o+s/14hPoRZX68ju0cg61XL2ylkdtIOCOViUUxJF87Naa9Zl89A==" saltValue="ey7HQ2TmfmhPQxHRRuklAA==" spinCount="100000" sheet="1" objects="1" scenarios="1" formatRows="0" insertRows="0" deleteRows="0" selectLockedCells="1"/>
   <mergeCells count="7">
     <mergeCell ref="A25:A32"/>
     <mergeCell ref="A5:C5"/>
@@ -3173,8 +3173,8 @@
       <c r="B12" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="C12" s="57"/>
-      <c r="D12" s="57"/>
+      <c r="C12" s="43"/>
+      <c r="D12" s="43"/>
     </row>
     <row r="13" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A13" s="11">
@@ -3183,18 +3183,18 @@
       <c r="B13" s="13" t="s">
         <v>53</v>
       </c>
-      <c r="C13" s="46"/>
-      <c r="D13" s="46"/>
+      <c r="C13" s="44"/>
+      <c r="D13" s="44"/>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="11">
         <v>3</v>
       </c>
-      <c r="B14" s="50" t="s">
+      <c r="B14" s="45" t="s">
         <v>37</v>
       </c>
-      <c r="C14" s="50"/>
-      <c r="D14" s="50"/>
+      <c r="C14" s="45"/>
+      <c r="D14" s="45"/>
     </row>
     <row r="15" spans="1:6" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="11" t="s">
@@ -3203,88 +3203,88 @@
       <c r="B15" s="14" t="s">
         <v>38</v>
       </c>
-      <c r="C15" s="57"/>
-      <c r="D15" s="57"/>
+      <c r="C15" s="43"/>
+      <c r="D15" s="43"/>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A16" s="41" t="s">
+      <c r="A16" s="49" t="s">
         <v>55</v>
       </c>
-      <c r="B16" s="45" t="s">
+      <c r="B16" s="53" t="s">
         <v>56</v>
       </c>
-      <c r="C16" s="50" t="s">
+      <c r="C16" s="45" t="s">
         <v>57</v>
       </c>
-      <c r="D16" s="50"/>
+      <c r="D16" s="45"/>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A17" s="41"/>
-      <c r="B17" s="45"/>
+      <c r="A17" s="49"/>
+      <c r="B17" s="53"/>
       <c r="C17" s="9"/>
       <c r="D17" s="8" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A18" s="41"/>
-      <c r="B18" s="45"/>
+      <c r="A18" s="49"/>
+      <c r="B18" s="53"/>
       <c r="C18" s="9"/>
       <c r="D18" s="8" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A19" s="41"/>
-      <c r="B19" s="45"/>
+      <c r="A19" s="49"/>
+      <c r="B19" s="53"/>
       <c r="C19" s="9"/>
       <c r="D19" s="8" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" s="41"/>
-      <c r="B20" s="45"/>
+      <c r="A20" s="49"/>
+      <c r="B20" s="53"/>
       <c r="C20" s="9"/>
       <c r="D20" s="8" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A21" s="41"/>
-      <c r="B21" s="45"/>
+      <c r="A21" s="49"/>
+      <c r="B21" s="53"/>
       <c r="C21" s="9"/>
       <c r="D21" s="8" t="s">
         <v>62</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A22" s="41"/>
-      <c r="B22" s="45"/>
-      <c r="C22" s="50" t="s">
+      <c r="A22" s="49"/>
+      <c r="B22" s="53"/>
+      <c r="C22" s="45" t="s">
         <v>63</v>
       </c>
-      <c r="D22" s="50"/>
+      <c r="D22" s="45"/>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A23" s="41"/>
-      <c r="B23" s="45"/>
+      <c r="A23" s="49"/>
+      <c r="B23" s="53"/>
       <c r="C23" s="9"/>
       <c r="D23" s="8" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A24" s="41"/>
-      <c r="B24" s="45"/>
+      <c r="A24" s="49"/>
+      <c r="B24" s="53"/>
       <c r="C24" s="9"/>
       <c r="D24" s="8" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A25" s="41"/>
-      <c r="B25" s="45"/>
+      <c r="A25" s="49"/>
+      <c r="B25" s="53"/>
       <c r="C25" s="9"/>
       <c r="D25" s="8" t="s">
         <v>62</v>
@@ -3294,11 +3294,11 @@
       <c r="A26" s="11" t="s">
         <v>64</v>
       </c>
-      <c r="B26" s="51" t="s">
+      <c r="B26" s="40" t="s">
         <v>65</v>
       </c>
-      <c r="C26" s="52"/>
-      <c r="D26" s="52"/>
+      <c r="C26" s="41"/>
+      <c r="D26" s="41"/>
     </row>
     <row r="27" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A27" s="11" t="s">
@@ -3307,8 +3307,8 @@
       <c r="B27" s="15" t="s">
         <v>67</v>
       </c>
-      <c r="C27" s="53"/>
-      <c r="D27" s="54"/>
+      <c r="C27" s="38"/>
+      <c r="D27" s="57"/>
     </row>
     <row r="28" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A28" s="11" t="s">
@@ -3317,18 +3317,18 @@
       <c r="B28" s="15" t="s">
         <v>69</v>
       </c>
-      <c r="C28" s="53"/>
-      <c r="D28" s="55"/>
+      <c r="C28" s="38"/>
+      <c r="D28" s="39"/>
     </row>
     <row r="29" spans="1:4" ht="28.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="11" t="s">
         <v>70</v>
       </c>
-      <c r="B29" s="51" t="s">
+      <c r="B29" s="40" t="s">
         <v>71</v>
       </c>
-      <c r="C29" s="52"/>
-      <c r="D29" s="52"/>
+      <c r="C29" s="41"/>
+      <c r="D29" s="41"/>
     </row>
     <row r="30" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A30" s="11" t="s">
@@ -3337,8 +3337,8 @@
       <c r="B30" s="15" t="s">
         <v>67</v>
       </c>
-      <c r="C30" s="56"/>
-      <c r="D30" s="56"/>
+      <c r="C30" s="42"/>
+      <c r="D30" s="42"/>
     </row>
     <row r="31" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A31" s="11" t="s">
@@ -3347,8 +3347,8 @@
       <c r="B31" s="15" t="s">
         <v>69</v>
       </c>
-      <c r="C31" s="46"/>
-      <c r="D31" s="46"/>
+      <c r="C31" s="44"/>
+      <c r="D31" s="44"/>
     </row>
     <row r="32" spans="1:4" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="11" t="s">
@@ -3357,8 +3357,8 @@
       <c r="B32" s="8" t="s">
         <v>75</v>
       </c>
-      <c r="C32" s="47"/>
-      <c r="D32" s="48"/>
+      <c r="C32" s="54"/>
+      <c r="D32" s="55"/>
     </row>
     <row r="33" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A33" s="11" t="s">
@@ -3367,8 +3367,8 @@
       <c r="B33" s="8" t="s">
         <v>77</v>
       </c>
-      <c r="C33" s="47"/>
-      <c r="D33" s="48"/>
+      <c r="C33" s="54"/>
+      <c r="D33" s="55"/>
     </row>
     <row r="34" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A34" s="11" t="s">
@@ -3377,8 +3377,8 @@
       <c r="B34" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="C34" s="49"/>
-      <c r="D34" s="49"/>
+      <c r="C34" s="56"/>
+      <c r="D34" s="56"/>
     </row>
     <row r="35" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A35" s="11" t="s">
@@ -3387,29 +3387,29 @@
       <c r="B35" s="16" t="s">
         <v>80</v>
       </c>
-      <c r="C35" s="48"/>
-      <c r="D35" s="48"/>
+      <c r="C35" s="55"/>
+      <c r="D35" s="55"/>
     </row>
     <row r="36" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A36" s="41" t="s">
+      <c r="A36" s="49" t="s">
         <v>81</v>
       </c>
-      <c r="B36" s="38" t="s">
+      <c r="B36" s="46" t="s">
         <v>82</v>
       </c>
-      <c r="C36" s="39"/>
-      <c r="D36" s="39"/>
-      <c r="E36" s="39"/>
-      <c r="F36" s="39"/>
-      <c r="G36" s="39"/>
-      <c r="H36" s="39"/>
-      <c r="I36" s="39"/>
-      <c r="J36" s="39"/>
-      <c r="K36" s="39"/>
-      <c r="L36" s="40"/>
+      <c r="C36" s="47"/>
+      <c r="D36" s="47"/>
+      <c r="E36" s="47"/>
+      <c r="F36" s="47"/>
+      <c r="G36" s="47"/>
+      <c r="H36" s="47"/>
+      <c r="I36" s="47"/>
+      <c r="J36" s="47"/>
+      <c r="K36" s="47"/>
+      <c r="L36" s="48"/>
     </row>
     <row r="37" spans="1:12" ht="105" x14ac:dyDescent="0.25">
-      <c r="A37" s="41"/>
+      <c r="A37" s="49"/>
       <c r="B37" s="15" t="s">
         <v>83</v>
       </c>
@@ -3445,7 +3445,7 @@
       </c>
     </row>
     <row r="38" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A38" s="41"/>
+      <c r="A38" s="49"/>
       <c r="B38" s="15">
         <v>1</v>
       </c>
@@ -3497,19 +3497,19 @@
       <c r="L39" s="29"/>
     </row>
     <row r="40" spans="1:12" ht="28.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="42">
+      <c r="A40" s="50">
         <v>9</v>
       </c>
-      <c r="B40" s="38" t="s">
+      <c r="B40" s="46" t="s">
         <v>92</v>
       </c>
-      <c r="C40" s="39"/>
-      <c r="D40" s="39"/>
-      <c r="E40" s="39"/>
-      <c r="F40" s="40"/>
+      <c r="C40" s="47"/>
+      <c r="D40" s="47"/>
+      <c r="E40" s="47"/>
+      <c r="F40" s="48"/>
     </row>
     <row r="41" spans="1:12" ht="45" x14ac:dyDescent="0.25">
-      <c r="A41" s="43"/>
+      <c r="A41" s="51"/>
       <c r="B41" s="8" t="s">
         <v>38</v>
       </c>
@@ -3527,7 +3527,7 @@
       </c>
     </row>
     <row r="42" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A42" s="44"/>
+      <c r="A42" s="52"/>
       <c r="B42" s="8">
         <v>1</v>
       </c>
@@ -3555,16 +3555,16 @@
       <c r="F43" s="20"/>
     </row>
     <row r="44" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A44" s="42">
+      <c r="A44" s="50">
         <v>10</v>
       </c>
-      <c r="B44" s="38" t="s">
+      <c r="B44" s="46" t="s">
         <v>98</v>
       </c>
-      <c r="C44" s="40"/>
+      <c r="C44" s="48"/>
     </row>
     <row r="45" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A45" s="43"/>
+      <c r="A45" s="51"/>
       <c r="B45" s="8" t="s">
         <v>99</v>
       </c>
@@ -3573,7 +3573,7 @@
       </c>
     </row>
     <row r="46" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A46" s="44"/>
+      <c r="A46" s="52"/>
       <c r="B46" s="8">
         <v>1</v>
       </c>
@@ -3635,17 +3635,8 @@
       <c r="B59" s="21"/>
     </row>
   </sheetData>
-  <sheetProtection formatRows="0" insertRows="0" deleteRows="0" selectLockedCells="1"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="ATUW55ixpZtA8LLP4oARyJvo05G6TzOdjXWfKjmgz/RhPwkI/Hix3RqyEC4mkD90l8WqdZLdT3/5Mi29bBBf8w==" saltValue="4/0ichV920yanSjJGZ+l5A==" spinCount="100000" sheet="1" objects="1" scenarios="1" formatRows="0" insertRows="0" deleteRows="0" selectLockedCells="1"/>
   <mergeCells count="25">
-    <mergeCell ref="C28:D28"/>
-    <mergeCell ref="B29:D29"/>
-    <mergeCell ref="C30:D30"/>
-    <mergeCell ref="A5:F5"/>
-    <mergeCell ref="C12:D12"/>
-    <mergeCell ref="C13:D13"/>
-    <mergeCell ref="B14:D14"/>
-    <mergeCell ref="C15:D15"/>
-    <mergeCell ref="C16:D16"/>
     <mergeCell ref="B40:F40"/>
     <mergeCell ref="B44:C44"/>
     <mergeCell ref="A16:A25"/>
@@ -3662,6 +3653,15 @@
     <mergeCell ref="C22:D22"/>
     <mergeCell ref="B26:D26"/>
     <mergeCell ref="C27:D27"/>
+    <mergeCell ref="C28:D28"/>
+    <mergeCell ref="B29:D29"/>
+    <mergeCell ref="C30:D30"/>
+    <mergeCell ref="A5:F5"/>
+    <mergeCell ref="C12:D12"/>
+    <mergeCell ref="C13:D13"/>
+    <mergeCell ref="B14:D14"/>
+    <mergeCell ref="C15:D15"/>
+    <mergeCell ref="C16:D16"/>
   </mergeCells>
   <dataValidations count="2">
     <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Неправильное значение" error="Номер корректировки - целое число в интервале от 0 до 99" sqref="B8">
@@ -3674,7 +3674,7 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" scale="40" orientation="landscape" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="35" orientation="landscape" r:id="rId1"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="2">

</xml_diff>